<commit_message>
#41 Updated LCSC MOQ Column removed.
</commit_message>
<xml_diff>
--- a/Deliverables/Interface_Board/BOM/NEW-6 Prototypes_Interface_Board.xlsx
+++ b/Deliverables/Interface_Board/BOM/NEW-6 Prototypes_Interface_Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ChristianRaun-EthercatDesign\Deliverables\Interface_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF979C34-0560-475B-8E10-1F732207B98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D3A7ABD-CD90-4A4A-93AF-082A2F30B043}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="256">
   <si>
     <t>Bill of Material (BOM) for Interface_Board</t>
   </si>
@@ -63,9 +63,6 @@
   </si>
   <si>
     <t>Value</t>
-  </si>
-  <si>
-    <t>LCSC/MOQ</t>
   </si>
   <si>
     <t>Quantity (Per Board)</t>
@@ -1474,7 +1471,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="180">
+  <cellXfs count="179">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1558,9 +1555,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1961,6 +1955,19 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1982,19 +1989,6 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2271,7 +2265,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD61"/>
+  <dimension ref="A1:AC61"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.140625" style="2" customWidth="1"/>
@@ -2284,31 +2278,29 @@
     <col min="8" max="8" width="15.28515625" style="2" customWidth="1"/>
     <col min="9" max="9" width="21.5703125" customWidth="1"/>
     <col min="10" max="10" width="7" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" customWidth="1"/>
-    <col min="12" max="12" width="21.85546875" customWidth="1"/>
-    <col min="13" max="13" width="14.140625" customWidth="1"/>
-    <col min="14" max="14" width="16.28515625" customWidth="1"/>
+    <col min="11" max="11" width="21.85546875" customWidth="1"/>
+    <col min="12" max="12" width="14.140625" customWidth="1"/>
+    <col min="13" max="13" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="16.5" thickBot="1">
-      <c r="A1" s="168" t="s">
+    <row r="1" spans="1:29" ht="16.5" thickBot="1">
+      <c r="A1" s="172" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="169"/>
-      <c r="C1" s="169"/>
-      <c r="D1" s="169"/>
-      <c r="E1" s="169"/>
-      <c r="F1" s="169"/>
-      <c r="G1" s="169"/>
-      <c r="H1" s="169"/>
-      <c r="I1" s="169"/>
-      <c r="J1" s="169"/>
-      <c r="K1" s="169"/>
-      <c r="L1" s="169"/>
-      <c r="M1" s="169"/>
-      <c r="N1" s="170"/>
-    </row>
-    <row r="2" spans="1:30" s="1" customFormat="1" ht="16.5" thickBot="1">
+      <c r="B1" s="173"/>
+      <c r="C1" s="173"/>
+      <c r="D1" s="173"/>
+      <c r="E1" s="173"/>
+      <c r="F1" s="173"/>
+      <c r="G1" s="173"/>
+      <c r="H1" s="173"/>
+      <c r="I1" s="173"/>
+      <c r="J1" s="173"/>
+      <c r="K1" s="173"/>
+      <c r="L1" s="173"/>
+      <c r="M1" s="174"/>
+    </row>
+    <row r="2" spans="1:29" s="1" customFormat="1" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -2342,15 +2334,13 @@
       <c r="K2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="M2" s="68" t="s">
-        <v>181</v>
-      </c>
-      <c r="N2" s="88" t="s">
+      <c r="L2" s="67" t="s">
         <v>180</v>
       </c>
+      <c r="M2" s="87" t="s">
+        <v>179</v>
+      </c>
+      <c r="N2"/>
       <c r="O2"/>
       <c r="P2"/>
       <c r="Q2"/>
@@ -2366,1835 +2356,1712 @@
       <c r="AA2"/>
       <c r="AB2"/>
       <c r="AC2"/>
-      <c r="AD2"/>
-    </row>
-    <row r="3" spans="1:30" ht="15.75" thickBot="1">
+    </row>
+    <row r="3" spans="1:29" ht="15.75" thickBot="1">
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="172" t="s">
+      <c r="B3" s="176" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="138" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="139" t="s">
+      <c r="D3" s="139" t="s">
+        <v>243</v>
+      </c>
+      <c r="E3" s="140" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="140" t="s">
-        <v>244</v>
-      </c>
-      <c r="E3" s="141" t="s">
+      <c r="F3" s="140" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="141" t="s">
+      <c r="G3" s="140" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="141" t="s">
+      <c r="H3" s="141" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="142" t="s">
-        <v>18</v>
-      </c>
-      <c r="I3" s="143" t="s">
+      <c r="I3" s="142" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="140" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="141" t="s">
+      <c r="K3" s="143">
+        <v>6</v>
+      </c>
+      <c r="L3" s="143">
+        <f>K3*6</f>
+        <v>36</v>
+      </c>
+      <c r="M3" s="144" t="s">
         <v>20</v>
       </c>
-      <c r="K3" s="144">
-        <v>50</v>
-      </c>
-      <c r="L3" s="144">
-        <v>6</v>
-      </c>
-      <c r="M3" s="144">
-        <f>L3*6</f>
-        <v>36</v>
-      </c>
-      <c r="N3" s="145" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:30" ht="15.75" thickBot="1">
+    </row>
+    <row r="4" spans="1:29" ht="15.75" thickBot="1">
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="173"/>
-      <c r="C4" s="146" t="s">
+      <c r="B4" s="177"/>
+      <c r="C4" s="145" t="s">
+        <v>208</v>
+      </c>
+      <c r="D4" s="146" t="s">
         <v>209</v>
       </c>
-      <c r="D4" s="147" t="s">
+      <c r="E4" s="131" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="132" t="s">
+        <v>207</v>
+      </c>
+      <c r="G4" s="132" t="s">
         <v>210</v>
       </c>
-      <c r="E4" s="132" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="133" t="s">
-        <v>208</v>
-      </c>
-      <c r="G4" s="133" t="s">
+      <c r="H4" s="147" t="s">
         <v>211</v>
       </c>
-      <c r="H4" s="148" t="s">
+      <c r="I4" s="148" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="132" t="s">
         <v>212</v>
       </c>
-      <c r="I4" s="149" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4" s="133" t="s">
-        <v>213</v>
-      </c>
-      <c r="K4" s="134">
+      <c r="K4" s="133">
+        <v>1</v>
+      </c>
+      <c r="L4" s="133">
+        <f t="shared" ref="L4:L6" si="0">K4*6</f>
+        <v>6</v>
+      </c>
+      <c r="M4" s="149" t="s">
         <v>20</v>
       </c>
-      <c r="L4" s="134">
-        <v>1</v>
-      </c>
-      <c r="M4" s="134">
-        <f t="shared" ref="M4:M6" si="0">L4*6</f>
-        <v>6</v>
-      </c>
-      <c r="N4" s="150" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:30" ht="15.75" thickBot="1">
+    </row>
+    <row r="5" spans="1:29" ht="15.75" thickBot="1">
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="173"/>
-      <c r="C5" s="146" t="s">
-        <v>218</v>
-      </c>
-      <c r="D5" s="147" t="s">
+      <c r="B5" s="177"/>
+      <c r="C5" s="145" t="s">
         <v>217</v>
       </c>
-      <c r="E5" s="132" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="133" t="s">
+      <c r="D5" s="146" t="s">
+        <v>216</v>
+      </c>
+      <c r="E5" s="131" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="132" t="s">
+        <v>213</v>
+      </c>
+      <c r="G5" s="132" t="s">
+        <v>210</v>
+      </c>
+      <c r="H5" s="147" t="s">
         <v>214</v>
       </c>
-      <c r="G5" s="133" t="s">
-        <v>211</v>
-      </c>
-      <c r="H5" s="148" t="s">
+      <c r="I5" s="148" t="s">
+        <v>18</v>
+      </c>
+      <c r="J5" s="132" t="s">
         <v>215</v>
       </c>
-      <c r="I5" s="149" t="s">
-        <v>19</v>
-      </c>
-      <c r="J5" s="133" t="s">
-        <v>216</v>
-      </c>
-      <c r="K5" s="134">
-        <v>50</v>
-      </c>
-      <c r="L5" s="134">
+      <c r="K5" s="133">
         <v>2</v>
       </c>
-      <c r="M5" s="134">
+      <c r="L5" s="133">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="N5" s="150" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M5" s="149" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" ht="15.75" thickBot="1">
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="173"/>
-      <c r="C6" s="176" t="s">
+      <c r="B6" s="177"/>
+      <c r="C6" s="168" t="s">
+        <v>246</v>
+      </c>
+      <c r="D6" s="146" t="s">
+        <v>245</v>
+      </c>
+      <c r="E6" s="131" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="167" t="s">
+        <v>244</v>
+      </c>
+      <c r="G6" s="131" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6" s="147" t="s">
         <v>247</v>
       </c>
-      <c r="D6" s="147" t="s">
-        <v>246</v>
-      </c>
-      <c r="E6" s="132" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="175" t="s">
-        <v>245</v>
-      </c>
-      <c r="G6" s="132" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="148" t="s">
+      <c r="I6" s="148" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="167" t="s">
         <v>248</v>
       </c>
-      <c r="I6" s="149" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6" s="175" t="s">
-        <v>249</v>
-      </c>
-      <c r="K6" s="134">
-        <v>30</v>
-      </c>
-      <c r="L6" s="134">
+      <c r="K6" s="133">
         <v>4</v>
       </c>
-      <c r="M6" s="134">
+      <c r="L6" s="133">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="N6" s="150" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M6" s="149" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" ht="15.75" thickBot="1">
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="173"/>
-      <c r="C7" s="35" t="s">
+      <c r="B7" s="177"/>
+      <c r="C7" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="D7" s="35" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="36" t="s">
+      <c r="E7" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="E7" s="37" t="s">
+      <c r="F7" s="35" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="36" t="s">
+      <c r="G7" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="G7" s="37" t="s">
+      <c r="H7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="I7" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="J7" s="36" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="J7" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="K7" s="11">
-        <v>10</v>
-      </c>
-      <c r="L7" s="8">
+      <c r="K7" s="8">
         <v>1</v>
       </c>
-      <c r="M7" s="11">
-        <f t="shared" ref="M7:M44" si="1">L7*6</f>
+      <c r="L7" s="11">
+        <f t="shared" ref="L7:L44" si="1">K7*6</f>
         <v>6</v>
       </c>
-      <c r="N7" s="83" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M7" s="82" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" ht="15.75" thickBot="1">
       <c r="A8" s="6">
         <v>6</v>
       </c>
-      <c r="B8" s="173"/>
-      <c r="C8" s="35" t="s">
+      <c r="B8" s="177"/>
+      <c r="C8" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="D8" s="36" t="s">
+      <c r="E8" s="36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="37" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="39" t="s">
+      <c r="G8" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="37" t="s">
+      <c r="H8" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="I8" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="J8" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="J8" s="37" t="s">
-        <v>35</v>
-      </c>
-      <c r="K8" s="11">
-        <v>100</v>
-      </c>
-      <c r="L8" s="8">
+      <c r="K8" s="8">
         <v>8</v>
       </c>
-      <c r="M8" s="11">
+      <c r="L8" s="11">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="N8" s="84" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M8" s="83" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" ht="15.75" thickBot="1">
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="173"/>
-      <c r="C9" s="151" t="s">
+      <c r="B9" s="177"/>
+      <c r="C9" s="150" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="132" t="s">
+        <v>232</v>
+      </c>
+      <c r="E9" s="131" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" s="161" t="s">
         <v>36</v>
       </c>
-      <c r="D9" s="133" t="s">
-        <v>233</v>
-      </c>
-      <c r="E9" s="132" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="162" t="s">
+      <c r="G9" s="148" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="149" t="s">
+      <c r="H9" s="76" t="s">
         <v>38</v>
       </c>
-      <c r="H9" s="77" t="s">
+      <c r="I9" s="131" t="s">
         <v>39</v>
       </c>
-      <c r="I9" s="132" t="s">
+      <c r="J9" s="131" t="s">
         <v>40</v>
       </c>
-      <c r="J9" s="132" t="s">
-        <v>41</v>
-      </c>
-      <c r="K9" s="134">
-        <v>50</v>
-      </c>
-      <c r="L9" s="77">
+      <c r="K9" s="76">
         <v>3</v>
       </c>
-      <c r="M9" s="134">
+      <c r="L9" s="133">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="N9" s="163" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M9" s="162" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" ht="15.75" thickBot="1">
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="173"/>
-      <c r="C10" s="40" t="s">
+      <c r="B10" s="177"/>
+      <c r="C10" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="35" t="s">
         <v>42</v>
       </c>
-      <c r="D10" s="36" t="s">
+      <c r="E10" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="41" t="s">
+      <c r="F10" s="35" t="s">
         <v>44</v>
       </c>
-      <c r="F10" s="36" t="s">
+      <c r="G10" s="41" t="s">
         <v>45</v>
       </c>
-      <c r="G10" s="42" t="s">
+      <c r="H10" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="I10" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="40" t="s">
         <v>47</v>
       </c>
-      <c r="I10" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="J10" s="41" t="s">
-        <v>48</v>
-      </c>
-      <c r="K10" s="11">
-        <v>10</v>
-      </c>
-      <c r="L10" s="28">
+      <c r="K10" s="28">
         <v>1</v>
       </c>
-      <c r="M10" s="11">
+      <c r="L10" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N10" s="85" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M10" s="84" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" ht="15.75" thickBot="1">
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="173"/>
-      <c r="C11" s="151" t="s">
+      <c r="B11" s="177"/>
+      <c r="C11" s="150" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="132" t="s">
+        <v>233</v>
+      </c>
+      <c r="E11" s="131" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="131" t="s">
         <v>49</v>
       </c>
-      <c r="D11" s="133" t="s">
-        <v>234</v>
-      </c>
-      <c r="E11" s="132" t="s">
-        <v>44</v>
-      </c>
-      <c r="F11" s="132" t="s">
+      <c r="G11" s="148" t="s">
+        <v>45</v>
+      </c>
+      <c r="H11" s="76" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="149" t="s">
-        <v>46</v>
-      </c>
-      <c r="H11" s="77" t="s">
-        <v>51</v>
-      </c>
-      <c r="I11" s="149" t="s">
-        <v>19</v>
-      </c>
-      <c r="J11" s="132" t="s">
-        <v>48</v>
-      </c>
-      <c r="K11" s="134">
+      <c r="I11" s="148" t="s">
+        <v>18</v>
+      </c>
+      <c r="J11" s="131" t="s">
+        <v>47</v>
+      </c>
+      <c r="K11" s="76">
+        <v>3</v>
+      </c>
+      <c r="L11" s="133">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+      <c r="M11" s="162" t="s">
         <v>20</v>
       </c>
-      <c r="L11" s="77">
-        <v>3</v>
-      </c>
-      <c r="M11" s="134">
-        <f t="shared" si="1"/>
-        <v>18</v>
-      </c>
-      <c r="N11" s="163" t="s">
-        <v>21</v>
-      </c>
-      <c r="O11" s="30"/>
-    </row>
-    <row r="12" spans="1:30" ht="15.75" thickBot="1">
+      <c r="N11" s="29"/>
+    </row>
+    <row r="12" spans="1:29" ht="15.75" thickBot="1">
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="173"/>
-      <c r="C12" s="78" t="s">
+      <c r="B12" s="177"/>
+      <c r="C12" s="77" t="s">
+        <v>161</v>
+      </c>
+      <c r="D12" s="68" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="60" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="60" t="s">
         <v>162</v>
       </c>
-      <c r="D12" s="69" t="s">
+      <c r="G12" s="41" t="s">
+        <v>25</v>
+      </c>
+      <c r="H12" s="75" t="s">
+        <v>240</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="E12" s="61" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="61" t="s">
-        <v>163</v>
-      </c>
-      <c r="G12" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="76" t="s">
-        <v>241</v>
-      </c>
-      <c r="I12" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="J12" s="41" t="s">
-        <v>53</v>
-      </c>
-      <c r="K12" s="11">
-        <v>20</v>
-      </c>
-      <c r="L12" s="12">
+      <c r="K12" s="12">
         <v>1</v>
       </c>
-      <c r="M12" s="11">
+      <c r="L12" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N12" s="86" t="s">
-        <v>21</v>
-      </c>
-      <c r="O12" s="30"/>
-    </row>
-    <row r="13" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M12" s="85" t="s">
+        <v>20</v>
+      </c>
+      <c r="N12" s="29"/>
+    </row>
+    <row r="13" spans="1:29" ht="15.75" thickBot="1">
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="173"/>
-      <c r="C13" s="40" t="s">
+      <c r="B13" s="177"/>
+      <c r="C13" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="D13" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="F13" s="35" t="s">
         <v>164</v>
       </c>
-      <c r="D13" s="36" t="s">
+      <c r="G13" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" s="75" t="s">
+        <v>241</v>
+      </c>
+      <c r="I13" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="J13" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="E13" s="41" t="s">
-        <v>24</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>165</v>
-      </c>
-      <c r="G13" s="42" t="s">
-        <v>17</v>
-      </c>
-      <c r="H13" s="76" t="s">
-        <v>242</v>
-      </c>
-      <c r="I13" s="38" t="s">
-        <v>19</v>
-      </c>
-      <c r="J13" s="41" t="s">
-        <v>55</v>
-      </c>
-      <c r="K13" s="11">
-        <v>10</v>
-      </c>
-      <c r="L13" s="12">
+      <c r="K13" s="12">
         <v>1</v>
       </c>
-      <c r="M13" s="11">
+      <c r="L13" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N13" s="86" t="s">
-        <v>21</v>
-      </c>
-      <c r="O13" s="31"/>
-    </row>
-    <row r="14" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M13" s="85" t="s">
+        <v>20</v>
+      </c>
+      <c r="N13" s="30"/>
+    </row>
+    <row r="14" spans="1:29" ht="15.75" thickBot="1">
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="174"/>
-      <c r="C14" s="43" t="s">
+      <c r="B14" s="178"/>
+      <c r="C14" s="42" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="43" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="44" t="s">
+      <c r="E14" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="45" t="s">
+      <c r="F14" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="F14" s="44" t="s">
+      <c r="G14" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="G14" s="46" t="s">
+      <c r="H14" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="H14" s="17" t="s">
+      <c r="I14" s="46" t="s">
+        <v>18</v>
+      </c>
+      <c r="J14" s="44" t="s">
         <v>61</v>
       </c>
-      <c r="I14" s="47" t="s">
-        <v>19</v>
-      </c>
-      <c r="J14" s="45" t="s">
-        <v>62</v>
-      </c>
-      <c r="K14" s="15">
-        <v>50</v>
-      </c>
-      <c r="L14" s="16">
+      <c r="K14" s="16">
         <v>1</v>
       </c>
-      <c r="M14" s="15">
+      <c r="L14" s="15">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N14" s="87" t="s">
-        <v>21</v>
-      </c>
-      <c r="O14" s="30"/>
-    </row>
-    <row r="15" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M14" s="86" t="s">
+        <v>20</v>
+      </c>
+      <c r="N14" s="29"/>
+    </row>
+    <row r="15" spans="1:29" ht="15.75" thickBot="1">
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="173" t="s">
+      <c r="B15" s="177" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" s="78" t="s">
         <v>63</v>
       </c>
-      <c r="C15" s="79" t="s">
+      <c r="D15" s="47" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="48" t="s">
+      <c r="E15" s="79" t="s">
         <v>65</v>
       </c>
-      <c r="E15" s="80" t="s">
+      <c r="F15" s="47" t="s">
         <v>66</v>
       </c>
-      <c r="F15" s="48" t="s">
+      <c r="G15" s="79" t="s">
         <v>67</v>
       </c>
-      <c r="G15" s="80" t="s">
+      <c r="H15" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="H15" s="20" t="s">
+      <c r="I15" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="80" t="s">
         <v>69</v>
       </c>
-      <c r="I15" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="J15" s="81" t="s">
-        <v>70</v>
-      </c>
-      <c r="K15" s="73">
-        <v>8</v>
-      </c>
-      <c r="L15" s="82">
+      <c r="K15" s="81">
         <v>1</v>
       </c>
-      <c r="M15" s="73">
+      <c r="L15" s="72">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N15" s="89" t="s">
-        <v>21</v>
-      </c>
-      <c r="O15" s="30"/>
-    </row>
-    <row r="16" spans="1:30" ht="15.75" thickBot="1">
+      <c r="M15" s="88" t="s">
+        <v>20</v>
+      </c>
+      <c r="N15" s="29"/>
+    </row>
+    <row r="16" spans="1:29" ht="15.75" thickBot="1">
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="173"/>
-      <c r="C16" s="151" t="s">
+      <c r="B16" s="177"/>
+      <c r="C16" s="150" t="s">
+        <v>221</v>
+      </c>
+      <c r="D16" s="151" t="s">
+        <v>220</v>
+      </c>
+      <c r="E16" s="132" t="s">
+        <v>219</v>
+      </c>
+      <c r="F16" s="132" t="s">
+        <v>218</v>
+      </c>
+      <c r="G16" s="132" t="s">
         <v>222</v>
       </c>
-      <c r="D16" s="152" t="s">
-        <v>221</v>
-      </c>
-      <c r="E16" s="133" t="s">
-        <v>220</v>
-      </c>
-      <c r="F16" s="133" t="s">
-        <v>219</v>
-      </c>
-      <c r="G16" s="133" t="s">
+      <c r="H16" s="152" t="s">
         <v>223</v>
       </c>
-      <c r="H16" s="153" t="s">
-        <v>224</v>
-      </c>
-      <c r="I16" s="154" t="s">
-        <v>19</v>
-      </c>
-      <c r="J16" s="154" t="s">
-        <v>70</v>
-      </c>
-      <c r="K16" s="134">
-        <v>50</v>
-      </c>
-      <c r="L16" s="77">
+      <c r="I16" s="153" t="s">
+        <v>18</v>
+      </c>
+      <c r="J16" s="153" t="s">
+        <v>69</v>
+      </c>
+      <c r="K16" s="76">
         <v>1</v>
       </c>
-      <c r="M16" s="134">
+      <c r="L16" s="133">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N16" s="136" t="s">
-        <v>21</v>
-      </c>
-      <c r="O16" s="30"/>
-    </row>
-    <row r="17" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M16" s="135" t="s">
+        <v>20</v>
+      </c>
+      <c r="N16" s="29"/>
+    </row>
+    <row r="17" spans="1:14" ht="15.75" thickBot="1">
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="173"/>
-      <c r="C17" s="146" t="s">
+      <c r="B17" s="177"/>
+      <c r="C17" s="145" t="s">
+        <v>237</v>
+      </c>
+      <c r="D17" s="151" t="s">
+        <v>236</v>
+      </c>
+      <c r="E17" s="132" t="s">
+        <v>235</v>
+      </c>
+      <c r="F17" s="132" t="s">
+        <v>234</v>
+      </c>
+      <c r="G17" s="132" t="s">
         <v>238</v>
       </c>
-      <c r="D17" s="152" t="s">
-        <v>237</v>
-      </c>
-      <c r="E17" s="133" t="s">
-        <v>236</v>
-      </c>
-      <c r="F17" s="133" t="s">
-        <v>235</v>
-      </c>
-      <c r="G17" s="133" t="s">
+      <c r="H17" s="152" t="s">
         <v>239</v>
       </c>
-      <c r="H17" s="153" t="s">
-        <v>240</v>
-      </c>
-      <c r="I17" s="154" t="s">
-        <v>19</v>
-      </c>
-      <c r="J17" s="154" t="s">
-        <v>70</v>
-      </c>
-      <c r="K17" s="134">
-        <v>10</v>
-      </c>
-      <c r="L17" s="77">
+      <c r="I17" s="153" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="153" t="s">
+        <v>69</v>
+      </c>
+      <c r="K17" s="76">
         <v>1</v>
       </c>
-      <c r="M17" s="134">
+      <c r="L17" s="133">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N17" s="136" t="s">
-        <v>21</v>
-      </c>
-      <c r="O17" s="30"/>
-    </row>
-    <row r="18" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M17" s="135" t="s">
+        <v>20</v>
+      </c>
+      <c r="N17" s="29"/>
+    </row>
+    <row r="18" spans="1:14" ht="15.75" thickBot="1">
       <c r="A18" s="6">
         <v>16</v>
       </c>
-      <c r="B18" s="173"/>
-      <c r="C18" s="75" t="s">
+      <c r="B18" s="177"/>
+      <c r="C18" s="74" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" s="100" t="s">
         <v>71</v>
       </c>
-      <c r="D18" s="101" t="s">
+      <c r="E18" s="104" t="s">
         <v>72</v>
       </c>
-      <c r="E18" s="105" t="s">
+      <c r="F18" s="100" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="101" t="s">
+      <c r="G18" s="104" t="s">
         <v>74</v>
       </c>
-      <c r="G18" s="105" t="s">
+      <c r="H18" s="101" t="s">
         <v>75</v>
       </c>
-      <c r="H18" s="102" t="s">
-        <v>76</v>
-      </c>
-      <c r="I18" s="102" t="s">
-        <v>19</v>
-      </c>
-      <c r="J18" s="106" t="s">
-        <v>70</v>
-      </c>
-      <c r="K18" s="98">
-        <v>20</v>
-      </c>
-      <c r="L18" s="107">
+      <c r="I18" s="101" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18" s="105" t="s">
+        <v>69</v>
+      </c>
+      <c r="K18" s="106">
         <v>1</v>
       </c>
-      <c r="M18" s="98">
+      <c r="L18" s="97">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N18" s="108" t="s">
-        <v>21</v>
-      </c>
-      <c r="O18" s="30"/>
-    </row>
-    <row r="19" spans="1:15" ht="16.5" thickBot="1">
+      <c r="M18" s="107" t="s">
+        <v>20</v>
+      </c>
+      <c r="N18" s="29"/>
+    </row>
+    <row r="19" spans="1:14" ht="16.5" thickBot="1">
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="167" t="s">
+      <c r="B19" s="166" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="108" t="s">
         <v>77</v>
       </c>
-      <c r="C19" s="109" t="s">
+      <c r="D19" s="109" t="s">
         <v>78</v>
       </c>
-      <c r="D19" s="110" t="s">
+      <c r="E19" s="109" t="s">
         <v>79</v>
       </c>
-      <c r="E19" s="110" t="s">
+      <c r="F19" s="109" t="s">
         <v>80</v>
       </c>
-      <c r="F19" s="110" t="s">
+      <c r="G19" s="110" t="s">
         <v>81</v>
       </c>
-      <c r="G19" s="111" t="s">
-        <v>82</v>
-      </c>
-      <c r="H19" s="111" t="s">
-        <v>19</v>
-      </c>
-      <c r="I19" s="110" t="s">
-        <v>19</v>
-      </c>
-      <c r="J19" s="111" t="s">
-        <v>70</v>
-      </c>
-      <c r="K19" s="103">
-        <v>7</v>
-      </c>
-      <c r="L19" s="103">
+      <c r="H19" s="110" t="s">
+        <v>18</v>
+      </c>
+      <c r="I19" s="109" t="s">
+        <v>18</v>
+      </c>
+      <c r="J19" s="110" t="s">
+        <v>69</v>
+      </c>
+      <c r="K19" s="102">
         <v>1</v>
       </c>
-      <c r="M19" s="66">
+      <c r="L19" s="65">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N19" s="104" t="s">
-        <v>21</v>
-      </c>
-      <c r="O19" s="30"/>
-    </row>
-    <row r="20" spans="1:15" ht="30.75" thickBot="1">
+      <c r="M19" s="103" t="s">
+        <v>20</v>
+      </c>
+      <c r="N19" s="29"/>
+    </row>
+    <row r="20" spans="1:14" ht="30.75" thickBot="1">
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="167" t="s">
+      <c r="B20" s="166" t="s">
+        <v>224</v>
+      </c>
+      <c r="C20" s="154" t="s">
+        <v>226</v>
+      </c>
+      <c r="D20" s="155" t="s">
         <v>225</v>
       </c>
-      <c r="C20" s="155" t="s">
+      <c r="E20" s="156" t="s">
         <v>227</v>
       </c>
-      <c r="D20" s="156" t="s">
-        <v>226</v>
-      </c>
-      <c r="E20" s="157" t="s">
+      <c r="F20" s="156" t="s">
         <v>228</v>
       </c>
-      <c r="F20" s="157" t="s">
+      <c r="G20" s="157" t="s">
         <v>229</v>
       </c>
-      <c r="G20" s="158" t="s">
+      <c r="H20" s="157" t="s">
         <v>230</v>
       </c>
-      <c r="H20" s="158" t="s">
+      <c r="I20" s="156" t="s">
         <v>231</v>
       </c>
-      <c r="I20" s="157" t="s">
-        <v>232</v>
-      </c>
-      <c r="J20" s="158" t="s">
-        <v>70</v>
-      </c>
-      <c r="K20" s="159">
-        <v>10</v>
+      <c r="J20" s="157" t="s">
+        <v>69</v>
+      </c>
+      <c r="K20" s="158">
+        <v>1</v>
       </c>
       <c r="L20" s="159">
-        <v>1</v>
-      </c>
-      <c r="M20" s="160">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N20" s="161" t="s">
-        <v>21</v>
-      </c>
-      <c r="O20" s="30"/>
-    </row>
-    <row r="21" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M20" s="160" t="s">
+        <v>20</v>
+      </c>
+      <c r="N20" s="29"/>
+    </row>
+    <row r="21" spans="1:14" ht="15.75" thickBot="1">
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="172" t="s">
-        <v>83</v>
-      </c>
-      <c r="C21" s="99" t="s">
+      <c r="B21" s="176" t="s">
+        <v>82</v>
+      </c>
+      <c r="C21" s="98" t="s">
+        <v>173</v>
+      </c>
+      <c r="D21" s="61" t="s">
         <v>174</v>
       </c>
-      <c r="D21" s="62" t="s">
+      <c r="E21" s="61" t="s">
         <v>175</v>
       </c>
-      <c r="E21" s="62" t="s">
+      <c r="F21" s="61" t="s">
+        <v>175</v>
+      </c>
+      <c r="G21" s="33" t="s">
         <v>176</v>
       </c>
-      <c r="F21" s="62" t="s">
-        <v>176</v>
-      </c>
-      <c r="G21" s="34" t="s">
+      <c r="H21" s="33" t="s">
         <v>177</v>
       </c>
-      <c r="H21" s="34" t="s">
-        <v>178</v>
-      </c>
-      <c r="I21" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="J21" s="34" t="s">
-        <v>70</v>
+      <c r="I21" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="J21" s="33" t="s">
+        <v>69</v>
       </c>
       <c r="K21" s="19">
-        <v>10</v>
-      </c>
-      <c r="L21" s="19">
         <v>1</v>
       </c>
-      <c r="M21" s="18">
+      <c r="L21" s="18">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N21" s="100" t="s">
-        <v>21</v>
-      </c>
-      <c r="O21" s="30"/>
-    </row>
-    <row r="22" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M21" s="99" t="s">
+        <v>20</v>
+      </c>
+      <c r="N21" s="29"/>
+    </row>
+    <row r="22" spans="1:14" ht="15.75" thickBot="1">
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="174"/>
-      <c r="C22" s="63" t="s">
+      <c r="B22" s="178"/>
+      <c r="C22" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="D22" s="63" t="s">
         <v>84</v>
       </c>
-      <c r="D22" s="64" t="s">
+      <c r="E22" s="63" t="s">
+        <v>43</v>
+      </c>
+      <c r="F22" s="63" t="s">
         <v>85</v>
       </c>
-      <c r="E22" s="64" t="s">
-        <v>44</v>
-      </c>
-      <c r="F22" s="64" t="s">
+      <c r="G22" s="63" t="s">
         <v>86</v>
       </c>
-      <c r="G22" s="64" t="s">
-        <v>87</v>
-      </c>
-      <c r="H22" s="65"/>
-      <c r="I22" s="65"/>
-      <c r="J22" s="64" t="s">
-        <v>70</v>
-      </c>
-      <c r="K22" s="65">
-        <v>7</v>
-      </c>
-      <c r="L22" s="65">
+      <c r="H22" s="64"/>
+      <c r="I22" s="64"/>
+      <c r="J22" s="63" t="s">
+        <v>69</v>
+      </c>
+      <c r="K22" s="64">
         <v>1</v>
       </c>
-      <c r="M22" s="15">
+      <c r="L22" s="15">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N22" s="67" t="s">
-        <v>88</v>
-      </c>
-      <c r="O22" s="30"/>
-    </row>
-    <row r="23" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M22" s="66" t="s">
+        <v>87</v>
+      </c>
+      <c r="N22" s="29"/>
+    </row>
+    <row r="23" spans="1:14" ht="15.75" thickBot="1">
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="172" t="s">
+      <c r="B23" s="176" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="138" t="s">
         <v>89</v>
       </c>
-      <c r="C23" s="139" t="s">
+      <c r="D23" s="163" t="s">
+        <v>186</v>
+      </c>
+      <c r="E23" s="140" t="s">
         <v>90</v>
       </c>
-      <c r="D23" s="164" t="s">
-        <v>187</v>
-      </c>
-      <c r="E23" s="141" t="s">
+      <c r="F23" s="140" t="s">
         <v>91</v>
       </c>
-      <c r="F23" s="141" t="s">
+      <c r="G23" s="142" t="s">
+        <v>59</v>
+      </c>
+      <c r="H23" s="164" t="s">
         <v>92</v>
       </c>
-      <c r="G23" s="143" t="s">
-        <v>60</v>
-      </c>
-      <c r="H23" s="165" t="s">
+      <c r="I23" s="140" t="s">
+        <v>18</v>
+      </c>
+      <c r="J23" s="140" t="s">
         <v>93</v>
       </c>
-      <c r="I23" s="141" t="s">
-        <v>19</v>
-      </c>
-      <c r="J23" s="141" t="s">
-        <v>94</v>
-      </c>
-      <c r="K23" s="144">
-        <v>100</v>
-      </c>
-      <c r="L23" s="144">
+      <c r="K23" s="143">
         <v>3</v>
       </c>
-      <c r="M23" s="144">
+      <c r="L23" s="143">
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="N23" s="166" t="s">
-        <v>21</v>
-      </c>
-      <c r="O23" s="30"/>
-    </row>
-    <row r="24" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M23" s="165" t="s">
+        <v>20</v>
+      </c>
+      <c r="N23" s="29"/>
+    </row>
+    <row r="24" spans="1:14" ht="15.75" thickBot="1">
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="173"/>
-      <c r="C24" s="72" t="s">
+      <c r="B24" s="177"/>
+      <c r="C24" s="71" t="s">
+        <v>165</v>
+      </c>
+      <c r="D24" s="60" t="s">
         <v>166</v>
       </c>
-      <c r="D24" s="61" t="s">
+      <c r="E24" s="60" t="s">
+        <v>90</v>
+      </c>
+      <c r="F24" s="60" t="s">
         <v>167</v>
       </c>
-      <c r="E24" s="61" t="s">
-        <v>91</v>
-      </c>
-      <c r="F24" s="61" t="s">
+      <c r="G24" s="37" t="s">
+        <v>155</v>
+      </c>
+      <c r="H24" s="75" t="s">
+        <v>242</v>
+      </c>
+      <c r="I24" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J24" s="73" t="s">
         <v>168</v>
       </c>
-      <c r="G24" s="38" t="s">
-        <v>156</v>
-      </c>
-      <c r="H24" s="76" t="s">
-        <v>243</v>
-      </c>
-      <c r="I24" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="J24" s="74" t="s">
-        <v>169</v>
-      </c>
       <c r="K24" s="7">
-        <v>100</v>
-      </c>
-      <c r="L24" s="7">
         <v>1</v>
       </c>
-      <c r="M24" s="11">
+      <c r="L24" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N24" s="90" t="s">
-        <v>179</v>
-      </c>
-      <c r="O24" s="30"/>
-    </row>
-    <row r="25" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M24" s="89" t="s">
+        <v>178</v>
+      </c>
+      <c r="N24" s="29"/>
+    </row>
+    <row r="25" spans="1:14" ht="15.75" thickBot="1">
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="173"/>
-      <c r="C25" s="128" t="s">
-        <v>195</v>
-      </c>
-      <c r="D25" s="129" t="s">
+      <c r="B25" s="177"/>
+      <c r="C25" s="127" t="s">
+        <v>194</v>
+      </c>
+      <c r="D25" s="128" t="s">
+        <v>187</v>
+      </c>
+      <c r="E25" s="70" t="s">
+        <v>90</v>
+      </c>
+      <c r="F25" s="129" t="s">
         <v>188</v>
       </c>
-      <c r="E25" s="71" t="s">
-        <v>91</v>
-      </c>
-      <c r="F25" s="130" t="s">
+      <c r="G25" s="129" t="s">
         <v>189</v>
       </c>
-      <c r="G25" s="130" t="s">
+      <c r="H25" s="130" t="s">
         <v>190</v>
       </c>
-      <c r="H25" s="131" t="s">
-        <v>191</v>
-      </c>
-      <c r="I25" s="132" t="s">
-        <v>19</v>
-      </c>
-      <c r="J25" s="133" t="s">
-        <v>201</v>
-      </c>
-      <c r="K25" s="134">
-        <v>20</v>
-      </c>
-      <c r="L25" s="134">
+      <c r="I25" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="J25" s="132" t="s">
+        <v>200</v>
+      </c>
+      <c r="K25" s="133">
         <v>1</v>
       </c>
-      <c r="M25" s="134">
+      <c r="L25" s="133">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N25" s="135" t="s">
-        <v>21</v>
-      </c>
-      <c r="O25" s="30"/>
-    </row>
-    <row r="26" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M25" s="134" t="s">
+        <v>20</v>
+      </c>
+      <c r="N25" s="29"/>
+    </row>
+    <row r="26" spans="1:14" ht="15.75" thickBot="1">
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="173"/>
-      <c r="C26" s="128" t="s">
-        <v>196</v>
-      </c>
-      <c r="D26" s="129" t="s">
+      <c r="B26" s="177"/>
+      <c r="C26" s="127" t="s">
+        <v>195</v>
+      </c>
+      <c r="D26" s="128" t="s">
+        <v>191</v>
+      </c>
+      <c r="E26" s="70" t="s">
+        <v>90</v>
+      </c>
+      <c r="F26" s="129" t="s">
         <v>192</v>
       </c>
-      <c r="E26" s="71" t="s">
-        <v>91</v>
-      </c>
-      <c r="F26" s="130" t="s">
+      <c r="G26" s="129" t="s">
+        <v>189</v>
+      </c>
+      <c r="H26" s="130" t="s">
         <v>193</v>
       </c>
-      <c r="G26" s="130" t="s">
-        <v>190</v>
-      </c>
-      <c r="H26" s="131" t="s">
-        <v>194</v>
-      </c>
-      <c r="I26" s="132" t="s">
-        <v>19</v>
-      </c>
-      <c r="J26" s="133" t="s">
-        <v>202</v>
-      </c>
-      <c r="K26" s="134">
-        <v>100</v>
-      </c>
-      <c r="L26" s="134">
+      <c r="I26" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="J26" s="132" t="s">
+        <v>201</v>
+      </c>
+      <c r="K26" s="133">
         <v>1</v>
       </c>
-      <c r="M26" s="134">
+      <c r="L26" s="133">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N26" s="136" t="s">
-        <v>21</v>
-      </c>
-      <c r="O26" s="30"/>
-    </row>
-    <row r="27" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M26" s="135" t="s">
+        <v>20</v>
+      </c>
+      <c r="N26" s="29"/>
+    </row>
+    <row r="27" spans="1:14" ht="15.75" thickBot="1">
       <c r="A27" s="6">
         <v>25</v>
       </c>
-      <c r="B27" s="173"/>
-      <c r="C27" s="128" t="s">
+      <c r="B27" s="177"/>
+      <c r="C27" s="127" t="s">
+        <v>197</v>
+      </c>
+      <c r="D27" s="128" t="s">
         <v>198</v>
       </c>
-      <c r="D27" s="129" t="s">
+      <c r="E27" s="132" t="s">
+        <v>90</v>
+      </c>
+      <c r="F27" s="136" t="s">
+        <v>196</v>
+      </c>
+      <c r="G27" s="129" t="s">
+        <v>189</v>
+      </c>
+      <c r="H27" s="137" t="s">
         <v>199</v>
       </c>
-      <c r="E27" s="133" t="s">
-        <v>91</v>
-      </c>
-      <c r="F27" s="137" t="s">
-        <v>197</v>
-      </c>
-      <c r="G27" s="130" t="s">
-        <v>190</v>
-      </c>
-      <c r="H27" s="138" t="s">
-        <v>200</v>
-      </c>
-      <c r="I27" s="132" t="s">
-        <v>19</v>
-      </c>
-      <c r="J27" s="133" t="s">
-        <v>203</v>
-      </c>
-      <c r="K27" s="134">
-        <v>100</v>
-      </c>
-      <c r="L27" s="134">
+      <c r="I27" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="J27" s="132" t="s">
+        <v>202</v>
+      </c>
+      <c r="K27" s="133">
         <v>1</v>
       </c>
-      <c r="M27" s="134">
+      <c r="L27" s="133">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N27" s="136" t="s">
-        <v>21</v>
-      </c>
-      <c r="O27" s="30"/>
-    </row>
-    <row r="28" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M27" s="135" t="s">
+        <v>20</v>
+      </c>
+      <c r="N27" s="29"/>
+    </row>
+    <row r="28" spans="1:14" ht="15.75" thickBot="1">
       <c r="A28" s="6">
         <v>26</v>
       </c>
-      <c r="B28" s="173"/>
-      <c r="C28" s="179" t="s">
-        <v>254</v>
-      </c>
-      <c r="D28" s="129" t="s">
-        <v>207</v>
-      </c>
-      <c r="E28" s="133" t="s">
-        <v>91</v>
-      </c>
-      <c r="F28" s="137" t="s">
+      <c r="B28" s="177"/>
+      <c r="C28" s="171" t="s">
+        <v>253</v>
+      </c>
+      <c r="D28" s="128" t="s">
+        <v>206</v>
+      </c>
+      <c r="E28" s="132" t="s">
+        <v>90</v>
+      </c>
+      <c r="F28" s="136" t="s">
+        <v>203</v>
+      </c>
+      <c r="G28" s="136" t="s">
+        <v>114</v>
+      </c>
+      <c r="H28" s="137" t="s">
         <v>204</v>
       </c>
-      <c r="G28" s="137" t="s">
-        <v>115</v>
-      </c>
-      <c r="H28" s="138" t="s">
+      <c r="I28" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="J28" s="132" t="s">
         <v>205</v>
       </c>
-      <c r="I28" s="132" t="s">
-        <v>19</v>
-      </c>
-      <c r="J28" s="133" t="s">
-        <v>206</v>
-      </c>
-      <c r="K28" s="134">
-        <v>50</v>
-      </c>
-      <c r="L28" s="134">
+      <c r="K28" s="133">
         <v>2</v>
       </c>
-      <c r="M28" s="134">
+      <c r="L28" s="133">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="N28" s="136" t="s">
-        <v>21</v>
-      </c>
-      <c r="O28" s="30"/>
-    </row>
-    <row r="29" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M28" s="135" t="s">
+        <v>20</v>
+      </c>
+      <c r="N28" s="29"/>
+    </row>
+    <row r="29" spans="1:14" ht="15.75" thickBot="1">
       <c r="A29" s="6">
         <v>27</v>
       </c>
-      <c r="B29" s="173"/>
-      <c r="C29" s="179" t="s">
-        <v>253</v>
-      </c>
-      <c r="D29" s="129" t="s">
-        <v>255</v>
-      </c>
-      <c r="E29" s="133" t="s">
-        <v>91</v>
-      </c>
-      <c r="F29" s="177" t="s">
+      <c r="B29" s="177"/>
+      <c r="C29" s="171" t="s">
+        <v>252</v>
+      </c>
+      <c r="D29" s="128" t="s">
+        <v>254</v>
+      </c>
+      <c r="E29" s="132" t="s">
+        <v>90</v>
+      </c>
+      <c r="F29" s="169" t="s">
+        <v>249</v>
+      </c>
+      <c r="G29" s="169" t="s">
+        <v>189</v>
+      </c>
+      <c r="H29" s="170" t="s">
         <v>250</v>
       </c>
-      <c r="G29" s="177" t="s">
-        <v>190</v>
-      </c>
-      <c r="H29" s="178" t="s">
+      <c r="I29" s="131" t="s">
+        <v>18</v>
+      </c>
+      <c r="J29" s="167" t="s">
         <v>251</v>
       </c>
-      <c r="I29" s="132" t="s">
-        <v>19</v>
-      </c>
-      <c r="J29" s="175" t="s">
-        <v>252</v>
-      </c>
-      <c r="K29" s="134">
-        <v>100</v>
-      </c>
-      <c r="L29" s="134">
+      <c r="K29" s="133">
         <v>2</v>
       </c>
-      <c r="M29" s="134">
+      <c r="L29" s="133">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="N29" s="136" t="s">
-        <v>21</v>
-      </c>
-      <c r="O29" s="30"/>
-    </row>
-    <row r="30" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M29" s="135" t="s">
+        <v>20</v>
+      </c>
+      <c r="N29" s="29"/>
+    </row>
+    <row r="30" spans="1:14" ht="15.75" thickBot="1">
       <c r="A30" s="6">
         <v>28</v>
       </c>
-      <c r="B30" s="173"/>
-      <c r="C30" s="50" t="s">
+      <c r="B30" s="177"/>
+      <c r="C30" s="49" t="s">
+        <v>94</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="E30" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="F30" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="E30" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F30" s="36" t="s">
+      <c r="G30" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="H30" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="G30" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="H30" s="13" t="s">
+      <c r="I30" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J30" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="I30" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="J30" s="36" t="s">
-        <v>99</v>
-      </c>
       <c r="K30" s="7">
-        <v>100</v>
-      </c>
-      <c r="L30" s="7">
         <v>2</v>
       </c>
-      <c r="M30" s="11">
+      <c r="L30" s="11">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="N30" s="91" t="s">
-        <v>21</v>
-      </c>
-      <c r="O30" s="30"/>
-    </row>
-    <row r="31" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M30" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="N30" s="29"/>
+    </row>
+    <row r="31" spans="1:14" ht="15.75" thickBot="1">
       <c r="A31" s="6">
         <v>29</v>
       </c>
-      <c r="B31" s="173"/>
-      <c r="C31" s="50" t="s">
+      <c r="B31" s="177"/>
+      <c r="C31" s="49" t="s">
+        <v>99</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="E31" s="35" t="s">
+        <v>90</v>
+      </c>
+      <c r="F31" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="D31" s="7" t="s">
-        <v>186</v>
-      </c>
-      <c r="E31" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F31" s="36" t="s">
+      <c r="G31" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="H31" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="G31" s="38" t="s">
-        <v>60</v>
-      </c>
-      <c r="H31" s="13" t="s">
+      <c r="I31" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J31" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="I31" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="J31" s="36" t="s">
-        <v>103</v>
-      </c>
       <c r="K31" s="7">
-        <v>100</v>
-      </c>
-      <c r="L31" s="7">
         <v>1</v>
       </c>
-      <c r="M31" s="11">
+      <c r="L31" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N31" s="91" t="s">
-        <v>21</v>
-      </c>
-      <c r="O31" s="30"/>
-    </row>
-    <row r="32" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M31" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="N31" s="29"/>
+    </row>
+    <row r="32" spans="1:14" ht="15.75" thickBot="1">
       <c r="A32" s="6">
         <v>30</v>
       </c>
-      <c r="B32" s="173"/>
-      <c r="C32" s="50" t="s">
+      <c r="B32" s="177"/>
+      <c r="C32" s="49" t="s">
+        <v>104</v>
+      </c>
+      <c r="D32" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="D32" s="36" t="s">
+      <c r="E32" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="F32" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="E32" s="36" t="s">
-        <v>104</v>
-      </c>
-      <c r="F32" s="39" t="s">
+      <c r="G32" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="G32" s="38" t="s">
+      <c r="H32" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="H32" s="13" t="s">
+      <c r="I32" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="I32" s="38" t="s">
+      <c r="J32" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="J32" s="36" t="s">
-        <v>111</v>
-      </c>
       <c r="K32" s="7">
-        <v>10</v>
-      </c>
-      <c r="L32" s="7">
         <v>1</v>
       </c>
-      <c r="M32" s="11">
+      <c r="L32" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N32" s="91" t="s">
-        <v>21</v>
-      </c>
-      <c r="O32" s="30"/>
-    </row>
-    <row r="33" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M32" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="N32" s="29"/>
+    </row>
+    <row r="33" spans="1:14" ht="15.75" thickBot="1">
       <c r="A33" s="6">
         <v>31</v>
       </c>
-      <c r="B33" s="173"/>
-      <c r="C33" s="50" t="s">
+      <c r="B33" s="177"/>
+      <c r="C33" s="49" t="s">
+        <v>111</v>
+      </c>
+      <c r="D33" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="D33" s="36" t="s">
+      <c r="E33" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="F33" s="35" t="s">
         <v>113</v>
       </c>
-      <c r="E33" s="36" t="s">
-        <v>24</v>
-      </c>
-      <c r="F33" s="36" t="s">
+      <c r="G33" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="G33" s="38" t="s">
+      <c r="H33" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="H33" s="13" t="s">
+      <c r="I33" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J33" s="35" t="s">
         <v>116</v>
       </c>
-      <c r="I33" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="J33" s="36" t="s">
-        <v>117</v>
-      </c>
       <c r="K33" s="7">
-        <v>100</v>
-      </c>
-      <c r="L33" s="7">
         <v>1</v>
       </c>
-      <c r="M33" s="11">
+      <c r="L33" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N33" s="91" t="s">
-        <v>21</v>
-      </c>
-      <c r="O33" s="30"/>
-    </row>
-    <row r="34" spans="1:15" s="1" customFormat="1" ht="15.75" thickBot="1">
+      <c r="M33" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="N33" s="29"/>
+    </row>
+    <row r="34" spans="1:14" s="1" customFormat="1" ht="15.75" thickBot="1">
       <c r="A34" s="6">
         <v>32</v>
       </c>
-      <c r="B34" s="174"/>
-      <c r="C34" s="51" t="s">
+      <c r="B34" s="178"/>
+      <c r="C34" s="50" t="s">
+        <v>117</v>
+      </c>
+      <c r="D34" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="E34" s="43" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" s="43" t="s">
         <v>119</v>
       </c>
-      <c r="E34" s="44" t="s">
-        <v>91</v>
-      </c>
-      <c r="F34" s="44" t="s">
+      <c r="G34" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="H34" s="17" t="s">
         <v>120</v>
       </c>
-      <c r="G34" s="47" t="s">
-        <v>60</v>
-      </c>
-      <c r="H34" s="17" t="s">
+      <c r="I34" s="43" t="s">
+        <v>18</v>
+      </c>
+      <c r="J34" s="43" t="s">
         <v>121</v>
       </c>
-      <c r="I34" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="J34" s="44" t="s">
-        <v>122</v>
-      </c>
-      <c r="K34" s="14">
-        <v>100</v>
-      </c>
-      <c r="L34" s="17">
+      <c r="K34" s="17">
         <v>8</v>
       </c>
-      <c r="M34" s="15">
+      <c r="L34" s="15">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
-      <c r="N34" s="113" t="s">
-        <v>21</v>
-      </c>
-      <c r="O34" s="32"/>
-    </row>
-    <row r="35" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M34" s="112" t="s">
+        <v>20</v>
+      </c>
+      <c r="N34" s="31"/>
+    </row>
+    <row r="35" spans="1:14" ht="15.75" thickBot="1">
       <c r="A35" s="6">
         <v>33</v>
       </c>
-      <c r="B35" s="173" t="s">
+      <c r="B35" s="177" t="s">
+        <v>122</v>
+      </c>
+      <c r="C35" s="118" t="s">
+        <v>184</v>
+      </c>
+      <c r="D35" s="126" t="s">
         <v>123</v>
       </c>
-      <c r="C35" s="119" t="s">
-        <v>185</v>
-      </c>
-      <c r="D35" s="127" t="s">
-        <v>124</v>
-      </c>
-      <c r="E35" s="112" t="s">
+      <c r="E35" s="111" t="s">
+        <v>181</v>
+      </c>
+      <c r="F35" s="120" t="s">
         <v>182</v>
       </c>
-      <c r="F35" s="121" t="s">
+      <c r="G35" s="121" t="s">
         <v>183</v>
       </c>
-      <c r="G35" s="122" t="s">
-        <v>184</v>
-      </c>
-      <c r="H35" s="123" t="s">
-        <v>19</v>
-      </c>
-      <c r="I35" s="120" t="s">
-        <v>19</v>
-      </c>
-      <c r="J35" s="123" t="s">
-        <v>70</v>
-      </c>
-      <c r="K35" s="124">
-        <v>7</v>
+      <c r="H35" s="122" t="s">
+        <v>18</v>
+      </c>
+      <c r="I35" s="119" t="s">
+        <v>18</v>
+      </c>
+      <c r="J35" s="122" t="s">
+        <v>69</v>
+      </c>
+      <c r="K35" s="123">
+        <v>1</v>
       </c>
       <c r="L35" s="124">
-        <v>1</v>
-      </c>
-      <c r="M35" s="125">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N35" s="126" t="s">
-        <v>21</v>
-      </c>
-      <c r="O35" s="30"/>
-    </row>
-    <row r="36" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M35" s="125" t="s">
+        <v>20</v>
+      </c>
+      <c r="N35" s="29"/>
+    </row>
+    <row r="36" spans="1:14" ht="15.75" thickBot="1">
       <c r="A36" s="6">
         <v>34</v>
       </c>
-      <c r="B36" s="173"/>
-      <c r="C36" s="50" t="s">
+      <c r="B36" s="177"/>
+      <c r="C36" s="49" t="s">
+        <v>124</v>
+      </c>
+      <c r="D36" s="35" t="s">
         <v>125</v>
       </c>
-      <c r="D36" s="36" t="s">
+      <c r="E36" s="35" t="s">
         <v>126</v>
       </c>
-      <c r="E36" s="36" t="s">
+      <c r="F36" s="35" t="s">
         <v>127</v>
       </c>
-      <c r="F36" s="36" t="s">
+      <c r="G36" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="G36" s="38" t="s">
+      <c r="H36" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="H36" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="I36" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="J36" s="38" t="s">
-        <v>70</v>
+      <c r="I36" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J36" s="37" t="s">
+        <v>69</v>
       </c>
       <c r="K36" s="13">
-        <v>6</v>
-      </c>
-      <c r="L36" s="13">
         <v>1</v>
       </c>
-      <c r="M36" s="11">
+      <c r="L36" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N36" s="91" t="s">
-        <v>21</v>
-      </c>
-      <c r="O36" s="30"/>
-    </row>
-    <row r="37" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M36" s="90" t="s">
+        <v>20</v>
+      </c>
+      <c r="N36" s="29"/>
+    </row>
+    <row r="37" spans="1:14" ht="15.75" thickBot="1">
       <c r="A37" s="6">
         <v>35</v>
       </c>
-      <c r="B37" s="173"/>
-      <c r="C37" s="114" t="s">
+      <c r="B37" s="177"/>
+      <c r="C37" s="113" t="s">
+        <v>169</v>
+      </c>
+      <c r="D37" s="114" t="s">
+        <v>130</v>
+      </c>
+      <c r="E37" s="114" t="s">
         <v>170</v>
       </c>
-      <c r="D37" s="115" t="s">
+      <c r="F37" s="115" t="s">
+        <v>172</v>
+      </c>
+      <c r="G37" s="100" t="s">
+        <v>171</v>
+      </c>
+      <c r="H37" s="96"/>
+      <c r="I37" s="100" t="s">
+        <v>18</v>
+      </c>
+      <c r="J37" s="101" t="s">
         <v>131</v>
       </c>
-      <c r="E37" s="115" t="s">
-        <v>171</v>
-      </c>
-      <c r="F37" s="116" t="s">
-        <v>173</v>
-      </c>
-      <c r="G37" s="101" t="s">
-        <v>172</v>
-      </c>
-      <c r="H37" s="97"/>
-      <c r="I37" s="101" t="s">
-        <v>19</v>
-      </c>
-      <c r="J37" s="102" t="s">
-        <v>132</v>
-      </c>
-      <c r="K37" s="97">
-        <v>6</v>
+      <c r="K37" s="96">
+        <v>1</v>
       </c>
       <c r="L37" s="97">
-        <v>1</v>
-      </c>
-      <c r="M37" s="98">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N37" s="117" t="s">
-        <v>88</v>
-      </c>
-      <c r="O37" s="30"/>
-    </row>
-    <row r="38" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M37" s="116" t="s">
+        <v>87</v>
+      </c>
+      <c r="N37" s="29"/>
+    </row>
+    <row r="38" spans="1:14" ht="15.75" thickBot="1">
       <c r="A38" s="6">
         <v>36</v>
       </c>
-      <c r="B38" s="172" t="s">
+      <c r="B38" s="176" t="s">
+        <v>132</v>
+      </c>
+      <c r="C38" s="51" t="s">
         <v>133</v>
       </c>
-      <c r="C38" s="52" t="s">
+      <c r="D38" s="52" t="s">
         <v>134</v>
       </c>
-      <c r="D38" s="53" t="s">
+      <c r="E38" s="52" t="s">
+        <v>255</v>
+      </c>
+      <c r="F38" s="52" t="s">
         <v>135</v>
       </c>
-      <c r="E38" s="53" t="s">
-        <v>256</v>
-      </c>
-      <c r="F38" s="53" t="s">
+      <c r="G38" s="52" t="s">
         <v>136</v>
       </c>
-      <c r="G38" s="53" t="s">
-        <v>137</v>
-      </c>
-      <c r="H38" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="I38" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="J38" s="53" t="s">
-        <v>70</v>
+      <c r="H38" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="I38" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="J38" s="52" t="s">
+        <v>69</v>
       </c>
       <c r="K38" s="22">
-        <v>100</v>
-      </c>
-      <c r="L38" s="22">
         <v>1</v>
       </c>
-      <c r="M38" s="18">
+      <c r="L38" s="18">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N38" s="118" t="s">
-        <v>138</v>
-      </c>
-      <c r="O38" s="30"/>
-    </row>
-    <row r="39" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M38" s="117" t="s">
+        <v>137</v>
+      </c>
+      <c r="N38" s="29"/>
+    </row>
+    <row r="39" spans="1:14" ht="15.75" thickBot="1">
       <c r="A39" s="6">
         <v>37</v>
       </c>
-      <c r="B39" s="173"/>
-      <c r="C39" s="54" t="s">
+      <c r="B39" s="177"/>
+      <c r="C39" s="53" t="s">
+        <v>138</v>
+      </c>
+      <c r="D39" s="54" t="s">
         <v>139</v>
       </c>
-      <c r="D39" s="55" t="s">
+      <c r="E39" s="54" t="s">
+        <v>43</v>
+      </c>
+      <c r="F39" s="54" t="s">
         <v>140</v>
       </c>
-      <c r="E39" s="55" t="s">
-        <v>44</v>
-      </c>
-      <c r="F39" s="55" t="s">
+      <c r="G39" s="54" t="s">
         <v>141</v>
       </c>
-      <c r="G39" s="55" t="s">
+      <c r="H39" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="I39" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="J39" s="55" t="s">
         <v>142</v>
       </c>
-      <c r="H39" s="55" t="s">
-        <v>19</v>
-      </c>
-      <c r="I39" s="55" t="s">
-        <v>19</v>
-      </c>
-      <c r="J39" s="56" t="s">
-        <v>143</v>
-      </c>
-      <c r="K39" s="29">
-        <v>12</v>
-      </c>
-      <c r="L39" s="23">
+      <c r="K39" s="23">
         <v>2</v>
       </c>
-      <c r="M39" s="11">
+      <c r="L39" s="11">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="N39" s="92" t="s">
-        <v>144</v>
-      </c>
-      <c r="O39" s="30"/>
-    </row>
-    <row r="40" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M39" s="91" t="s">
+        <v>143</v>
+      </c>
+      <c r="N39" s="29"/>
+    </row>
+    <row r="40" spans="1:14" ht="15.75" thickBot="1">
       <c r="A40" s="6">
         <v>38</v>
       </c>
-      <c r="B40" s="173"/>
-      <c r="C40" s="54" t="s">
+      <c r="B40" s="177"/>
+      <c r="C40" s="53" t="s">
+        <v>144</v>
+      </c>
+      <c r="D40" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="D40" s="55" t="s">
+      <c r="E40" s="54" t="s">
+        <v>43</v>
+      </c>
+      <c r="F40" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="E40" s="55" t="s">
-        <v>44</v>
-      </c>
-      <c r="F40" s="55" t="s">
-        <v>147</v>
-      </c>
-      <c r="G40" s="55" t="s">
-        <v>137</v>
-      </c>
-      <c r="H40" s="55" t="s">
-        <v>19</v>
-      </c>
-      <c r="I40" s="55" t="s">
-        <v>19</v>
-      </c>
-      <c r="J40" s="56" t="s">
-        <v>70</v>
-      </c>
-      <c r="K40" s="29">
-        <v>10</v>
-      </c>
-      <c r="L40" s="23">
+      <c r="G40" s="54" t="s">
+        <v>136</v>
+      </c>
+      <c r="H40" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="I40" s="54" t="s">
+        <v>18</v>
+      </c>
+      <c r="J40" s="55" t="s">
+        <v>69</v>
+      </c>
+      <c r="K40" s="23">
         <v>1</v>
       </c>
-      <c r="M40" s="11">
+      <c r="L40" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N40" s="92" t="s">
-        <v>138</v>
-      </c>
-      <c r="O40" s="30"/>
-    </row>
-    <row r="41" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M40" s="91" t="s">
+        <v>137</v>
+      </c>
+      <c r="N40" s="29"/>
+    </row>
+    <row r="41" spans="1:14" ht="15.75" thickBot="1">
       <c r="A41" s="6">
         <v>39</v>
       </c>
-      <c r="B41" s="173"/>
+      <c r="B41" s="177"/>
       <c r="C41" s="21" t="s">
+        <v>147</v>
+      </c>
+      <c r="D41" s="35" t="s">
         <v>148</v>
       </c>
-      <c r="D41" s="36" t="s">
+      <c r="E41" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="F41" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="E41" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="F41" s="36" t="s">
+      <c r="G41" s="35" t="s">
         <v>150</v>
       </c>
-      <c r="G41" s="36" t="s">
-        <v>151</v>
-      </c>
-      <c r="H41" s="36" t="s">
-        <v>150</v>
-      </c>
-      <c r="I41" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="J41" s="38" t="s">
-        <v>143</v>
-      </c>
-      <c r="K41" s="13">
-        <v>20</v>
-      </c>
-      <c r="L41" s="7">
+      <c r="H41" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I41" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J41" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="K41" s="7">
         <v>1</v>
       </c>
-      <c r="M41" s="11">
+      <c r="L41" s="11">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="N41" s="93" t="s">
-        <v>21</v>
-      </c>
-      <c r="O41" s="30"/>
-    </row>
-    <row r="42" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M41" s="92" t="s">
+        <v>20</v>
+      </c>
+      <c r="N41" s="29"/>
+    </row>
+    <row r="42" spans="1:14" ht="15.75" thickBot="1">
       <c r="A42" s="6">
         <v>40</v>
       </c>
-      <c r="B42" s="173"/>
-      <c r="C42" s="50" t="s">
+      <c r="B42" s="177"/>
+      <c r="C42" s="49" t="s">
+        <v>151</v>
+      </c>
+      <c r="D42" s="35" t="s">
         <v>152</v>
       </c>
-      <c r="D42" s="36" t="s">
+      <c r="E42" s="35" t="s">
         <v>153</v>
       </c>
-      <c r="E42" s="36" t="s">
+      <c r="F42" s="35" t="s">
         <v>154</v>
       </c>
-      <c r="F42" s="36" t="s">
+      <c r="G42" s="35" t="s">
         <v>155</v>
       </c>
-      <c r="G42" s="36" t="s">
+      <c r="H42" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="H42" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="I42" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="J42" s="38" t="s">
-        <v>70</v>
+      <c r="I42" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="J42" s="37" t="s">
+        <v>69</v>
       </c>
       <c r="K42" s="13">
-        <v>15</v>
-      </c>
-      <c r="L42" s="13">
         <v>2</v>
       </c>
-      <c r="M42" s="11">
+      <c r="L42" s="11">
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="N42" s="94" t="s">
-        <v>21</v>
-      </c>
-      <c r="O42" s="30"/>
-    </row>
-    <row r="43" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M42" s="93" t="s">
+        <v>20</v>
+      </c>
+      <c r="N42" s="29"/>
+    </row>
+    <row r="43" spans="1:14" ht="15.75" thickBot="1">
       <c r="A43" s="6">
         <v>41</v>
       </c>
-      <c r="B43" s="173"/>
-      <c r="C43" s="57" t="s">
+      <c r="B43" s="177"/>
+      <c r="C43" s="56" t="s">
+        <v>157</v>
+      </c>
+      <c r="D43" s="24"/>
+      <c r="E43" s="57" t="s">
         <v>158</v>
       </c>
-      <c r="D43" s="24"/>
-      <c r="E43" s="58" t="s">
-        <v>159</v>
-      </c>
       <c r="F43" s="24" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G43" s="24"/>
       <c r="H43" s="24"/>
       <c r="I43" s="24"/>
       <c r="J43" s="24"/>
-      <c r="K43" s="24"/>
-      <c r="L43" s="24">
+      <c r="K43" s="24">
         <v>5</v>
       </c>
-      <c r="M43" s="11">
+      <c r="L43" s="11">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="N43" s="95" t="s">
-        <v>19</v>
-      </c>
-      <c r="O43" s="30"/>
-    </row>
-    <row r="44" spans="1:15" ht="15.75" thickBot="1">
+      <c r="M43" s="94" t="s">
+        <v>18</v>
+      </c>
+      <c r="N43" s="29"/>
+    </row>
+    <row r="44" spans="1:14" ht="15.75" thickBot="1">
       <c r="A44" s="6">
         <v>42</v>
       </c>
-      <c r="B44" s="174"/>
-      <c r="C44" s="59" t="s">
+      <c r="B44" s="178"/>
+      <c r="C44" s="58" t="s">
+        <v>159</v>
+      </c>
+      <c r="D44" s="25"/>
+      <c r="E44" s="59" t="s">
         <v>160</v>
       </c>
-      <c r="D44" s="25"/>
-      <c r="E44" s="60" t="s">
-        <v>161</v>
-      </c>
       <c r="F44" s="25" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G44" s="25"/>
       <c r="H44" s="25"/>
       <c r="I44" s="25"/>
       <c r="J44" s="25"/>
-      <c r="K44" s="25"/>
-      <c r="L44" s="25">
+      <c r="K44" s="25">
         <v>5</v>
       </c>
-      <c r="M44" s="15">
+      <c r="L44" s="15">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="N44" s="96" t="s">
-        <v>19</v>
-      </c>
-      <c r="O44" s="30"/>
-    </row>
-    <row r="45" spans="1:15" ht="16.5" thickBot="1">
+      <c r="M44" s="95" t="s">
+        <v>18</v>
+      </c>
+      <c r="N44" s="29"/>
+    </row>
+    <row r="45" spans="1:14" ht="16.5" thickBot="1">
       <c r="A45"/>
       <c r="C45" s="26"/>
       <c r="D45" s="26"/>
@@ -4204,13 +4071,12 @@
       <c r="H45" s="26"/>
       <c r="I45" s="26"/>
       <c r="J45" s="26"/>
-      <c r="K45" s="26"/>
-      <c r="L45" s="171"/>
-      <c r="M45" s="171"/>
-      <c r="N45" s="171"/>
-      <c r="O45" s="30"/>
-    </row>
-    <row r="46" spans="1:15">
+      <c r="K45" s="175"/>
+      <c r="L45" s="175"/>
+      <c r="M45" s="175"/>
+      <c r="N45" s="29"/>
+    </row>
+    <row r="46" spans="1:14">
       <c r="A46"/>
       <c r="C46" s="26"/>
       <c r="D46" s="26"/>
@@ -4220,72 +4086,71 @@
       <c r="H46" s="26"/>
       <c r="I46" s="26"/>
       <c r="J46" s="26"/>
-      <c r="K46" s="26"/>
-      <c r="O46" s="30"/>
-    </row>
-    <row r="47" spans="1:15">
+      <c r="N46" s="29"/>
+    </row>
+    <row r="47" spans="1:14">
       <c r="A47"/>
-      <c r="O47" s="30"/>
-    </row>
-    <row r="48" spans="1:15">
+      <c r="N47" s="29"/>
+    </row>
+    <row r="48" spans="1:14">
       <c r="A48"/>
-      <c r="O48" s="30"/>
-    </row>
-    <row r="49" spans="1:15">
+      <c r="N48" s="29"/>
+    </row>
+    <row r="49" spans="1:14">
       <c r="A49"/>
-      <c r="O49" s="30"/>
-    </row>
-    <row r="50" spans="1:15">
+      <c r="N49" s="29"/>
+    </row>
+    <row r="50" spans="1:14">
       <c r="A50"/>
-      <c r="O50" s="30"/>
-    </row>
-    <row r="51" spans="1:15">
+      <c r="N50" s="29"/>
+    </row>
+    <row r="51" spans="1:14">
       <c r="A51"/>
-      <c r="O51" s="30"/>
-    </row>
-    <row r="52" spans="1:15">
+      <c r="N51" s="29"/>
+    </row>
+    <row r="52" spans="1:14">
       <c r="A52"/>
-      <c r="O52" s="30"/>
-    </row>
-    <row r="53" spans="1:15">
+      <c r="N52" s="29"/>
+    </row>
+    <row r="53" spans="1:14">
       <c r="A53"/>
-      <c r="O53" s="30"/>
-    </row>
-    <row r="54" spans="1:15" ht="15.75" customHeight="1">
+      <c r="N53" s="29"/>
+    </row>
+    <row r="54" spans="1:14" ht="15.75" customHeight="1">
       <c r="A54"/>
-      <c r="N54" s="70"/>
-      <c r="O54" s="30"/>
-    </row>
-    <row r="55" spans="1:15">
+      <c r="M54" s="69"/>
+      <c r="N54" s="29"/>
+    </row>
+    <row r="55" spans="1:14">
       <c r="A55"/>
-      <c r="O55" s="30"/>
-    </row>
-    <row r="56" spans="1:15">
+      <c r="N55" s="29"/>
+    </row>
+    <row r="56" spans="1:14">
       <c r="A56"/>
-      <c r="O56" s="30"/>
-    </row>
-    <row r="57" spans="1:15">
+      <c r="N56" s="29"/>
+    </row>
+    <row r="57" spans="1:14">
       <c r="A57"/>
-      <c r="O57" s="30"/>
-    </row>
-    <row r="58" spans="1:15">
+      <c r="N57" s="29"/>
+    </row>
+    <row r="58" spans="1:14">
       <c r="A58"/>
-      <c r="O58" s="30"/>
-    </row>
-    <row r="59" spans="1:15">
+      <c r="N58" s="29"/>
+    </row>
+    <row r="59" spans="1:14">
       <c r="A59"/>
-      <c r="O59" s="30"/>
-    </row>
-    <row r="60" spans="1:15">
+      <c r="N59" s="29"/>
+    </row>
+    <row r="60" spans="1:14">
       <c r="H60" s="27"/>
     </row>
-    <row r="61" spans="1:15">
+    <row r="61" spans="1:14">
       <c r="H61" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A1:N1"/>
-    <mergeCell ref="L45:N45"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="K45:M45"/>
     <mergeCell ref="B3:B14"/>
     <mergeCell ref="B15:B18"/>
     <mergeCell ref="B23:B34"/>
@@ -4294,7 +4159,7 @@
     <mergeCell ref="B21:B22"/>
   </mergeCells>
   <phoneticPr fontId="21" type="noConversion"/>
-  <conditionalFormatting sqref="N22">
+  <conditionalFormatting sqref="M22">
     <cfRule type="dataBar" priority="38">
       <dataBar>
         <cfvo type="min"/>
@@ -4308,7 +4173,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L38:M38">
+  <conditionalFormatting sqref="K38:L38">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -4320,7 +4185,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L43">
+  <conditionalFormatting sqref="K43">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -4342,7 +4207,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L44">
+  <conditionalFormatting sqref="K44">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
@@ -4364,7 +4229,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N3:N7">
+  <conditionalFormatting sqref="M3:M7">
     <cfRule type="dataBar" priority="40">
       <dataBar>
         <cfvo type="min"/>
@@ -4378,7 +4243,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N34">
+  <conditionalFormatting sqref="M34">
     <cfRule type="dataBar" priority="37">
       <dataBar>
         <cfvo type="min"/>
@@ -4392,7 +4257,7 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L13:L37 L42 M3:M44">
+  <conditionalFormatting sqref="K13:K37 K42 L3:L44">
     <cfRule type="colorScale" priority="50">
       <colorScale>
         <cfvo type="min"/>
@@ -4404,7 +4269,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L9:L12">
+  <conditionalFormatting sqref="K9:K12">
     <cfRule type="colorScale" priority="51">
       <colorScale>
         <cfvo type="min"/>
@@ -4416,7 +4281,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:M44">
+  <conditionalFormatting sqref="K3:L44">
     <cfRule type="colorScale" priority="61">
       <colorScale>
         <cfvo type="min"/>
@@ -4429,44 +4294,44 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="N11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="N14" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="N15" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="N18" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="N23" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="N30" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="N31" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="N33" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="N34" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="N36" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="N42" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="N9" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="N32" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="N3" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="N7" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="N8" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="N38" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="N40" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="N19" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="N41" r:id="rId21" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="N21" r:id="rId22" xr:uid="{5EAF2F70-555A-4B25-966F-95095861DC0E}"/>
-    <hyperlink ref="N24" r:id="rId23" xr:uid="{6B884554-8BB6-4BF7-8096-D834E9729A06}"/>
-    <hyperlink ref="N12" r:id="rId24" xr:uid="{44B658D6-BFFD-46B9-B230-29405BAF9534}"/>
-    <hyperlink ref="N13" r:id="rId25" xr:uid="{367FEFFE-61E8-47BB-BCCA-FD3358349566}"/>
-    <hyperlink ref="N35" r:id="rId26" xr:uid="{D1D06D79-D259-47BA-BC7F-8742EAB7848C}"/>
-    <hyperlink ref="N25" r:id="rId27" xr:uid="{5545F658-0692-42E9-BD6F-76E0A6B030B0}"/>
-    <hyperlink ref="N27" r:id="rId28" xr:uid="{168ECF43-5CE3-4702-A056-8FA8BBC47676}"/>
-    <hyperlink ref="N26" r:id="rId29" xr:uid="{EA5E5506-441F-4FE0-B453-D92044CD3CD6}"/>
-    <hyperlink ref="N28" r:id="rId30" xr:uid="{8D8C1B68-82FF-4307-AFCC-0412DDB5B0BE}"/>
-    <hyperlink ref="N4" r:id="rId31" xr:uid="{2EF0B57E-A4CF-4AC0-9358-948CDF39D8B4}"/>
-    <hyperlink ref="N5" r:id="rId32" xr:uid="{ECCB4777-894F-4969-BB30-3BB1C2789276}"/>
+    <hyperlink ref="M10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="M11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="M14" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="M15" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="M18" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="M23" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="M30" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="M31" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="M33" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="M34" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="M36" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="M42" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="M9" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="M32" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="M3" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="M7" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="M8" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="M38" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="M40" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="M19" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="M41" r:id="rId21" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="M21" r:id="rId22" xr:uid="{5EAF2F70-555A-4B25-966F-95095861DC0E}"/>
+    <hyperlink ref="M24" r:id="rId23" xr:uid="{6B884554-8BB6-4BF7-8096-D834E9729A06}"/>
+    <hyperlink ref="M12" r:id="rId24" xr:uid="{44B658D6-BFFD-46B9-B230-29405BAF9534}"/>
+    <hyperlink ref="M13" r:id="rId25" xr:uid="{367FEFFE-61E8-47BB-BCCA-FD3358349566}"/>
+    <hyperlink ref="M35" r:id="rId26" xr:uid="{D1D06D79-D259-47BA-BC7F-8742EAB7848C}"/>
+    <hyperlink ref="M25" r:id="rId27" xr:uid="{5545F658-0692-42E9-BD6F-76E0A6B030B0}"/>
+    <hyperlink ref="M27" r:id="rId28" xr:uid="{168ECF43-5CE3-4702-A056-8FA8BBC47676}"/>
+    <hyperlink ref="M26" r:id="rId29" xr:uid="{EA5E5506-441F-4FE0-B453-D92044CD3CD6}"/>
+    <hyperlink ref="M28" r:id="rId30" xr:uid="{8D8C1B68-82FF-4307-AFCC-0412DDB5B0BE}"/>
+    <hyperlink ref="M4" r:id="rId31" xr:uid="{2EF0B57E-A4CF-4AC0-9358-948CDF39D8B4}"/>
+    <hyperlink ref="M5" r:id="rId32" xr:uid="{ECCB4777-894F-4969-BB30-3BB1C2789276}"/>
     <hyperlink ref="C16" r:id="rId33" xr:uid="{44A99C6C-4AC4-4D03-96BE-D592031C9536}"/>
-    <hyperlink ref="N16" r:id="rId34" xr:uid="{1A7B0E41-616E-45F1-BF6C-4CBB22A55EC6}"/>
-    <hyperlink ref="N20" r:id="rId35" xr:uid="{0E9DC705-3503-4FA0-87A9-DF2A5B60045D}"/>
-    <hyperlink ref="N17" r:id="rId36" xr:uid="{E7A9FE43-2492-4F96-944F-8153D9DD3BC5}"/>
-    <hyperlink ref="N6" r:id="rId37" xr:uid="{C6B216F8-5775-4357-B676-8FC9F8808265}"/>
-    <hyperlink ref="N29" r:id="rId38" xr:uid="{A2E7CF78-849E-4B20-A638-AA9D3B8EC8EE}"/>
+    <hyperlink ref="M16" r:id="rId34" xr:uid="{1A7B0E41-616E-45F1-BF6C-4CBB22A55EC6}"/>
+    <hyperlink ref="M20" r:id="rId35" xr:uid="{0E9DC705-3503-4FA0-87A9-DF2A5B60045D}"/>
+    <hyperlink ref="M17" r:id="rId36" xr:uid="{E7A9FE43-2492-4F96-944F-8153D9DD3BC5}"/>
+    <hyperlink ref="M6" r:id="rId37" xr:uid="{C6B216F8-5775-4357-B676-8FC9F8808265}"/>
+    <hyperlink ref="M29" r:id="rId38" xr:uid="{A2E7CF78-849E-4B20-A638-AA9D3B8EC8EE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId39"/>
@@ -4484,7 +4349,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>N22</xm:sqref>
+          <xm:sqref>M22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{94E20060-874B-439F-8FDA-33B3DD39FFE6}">
@@ -4497,7 +4362,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>N3:N7</xm:sqref>
+          <xm:sqref>M3:M7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{DBB933A5-5D45-42AE-8D8B-F05439EF033D}">
@@ -4510,7 +4375,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>N34</xm:sqref>
+          <xm:sqref>M34</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>